<commit_message>
Bản vá bug của summon
</commit_message>
<xml_diff>
--- a/Assets/Document/02_Data/a_CardsData.xlsx
+++ b/Assets/Document/02_Data/a_CardsData.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspaces\specialized-essays\AutoChess\Assets\Resources\Document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspaces\specialized-essays\AutoChess\Assets\Document\02_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB145BA1-1AEB-4847-AA18-8C4324B03F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DEF3E5-C938-4188-ADE3-EE4FEB83D547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{4D4D67B0-B191-4148-8DB5-7E5E04C9AFB3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{4D4D67B0-B191-4148-8DB5-7E5E04C9AFB3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Niles" sheetId="1" r:id="rId1"/>
+    <sheet name="Babylon" sheetId="2" r:id="rId2"/>
+    <sheet name="Spells" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="154">
   <si>
     <t>Tribe</t>
   </si>
@@ -195,178 +196,320 @@
     <t>Taunt; Reborn</t>
   </si>
   <si>
-    <t>Tên Unit</t>
-  </si>
-  <si>
-    <t>Trigger (Khi nào?)</t>
-  </si>
-  <si>
-    <t>Target (Ai?)</t>
-  </si>
-  <si>
-    <t>Effect (Làm gì?)</t>
-  </si>
-  <si>
-    <t>Điểm cần lưu ý</t>
-  </si>
-  <si>
-    <t>OnAllyDemise</t>
-  </si>
-  <si>
-    <t>LowestHealthAlly</t>
-  </si>
-  <si>
-    <r>
-      <t>GiveBuff</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Reborn)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Cần thêm biến </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF444746"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>LimitPerBattle = 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>OnAllySummon</t>
-  </si>
-  <si>
-    <t>LastSummoned</t>
-  </si>
-  <si>
-    <t>Destroy</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Phần Demise: dùng </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF444746"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>Effect: Summon</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>StartOfBattle</t>
-  </si>
-  <si>
-    <t>LeftAlly</t>
-  </si>
-  <si>
-    <t>TriggerAbility</t>
-  </si>
-  <si>
-    <t>TargetID cần xác định theo vị trí Board (-1 slot).</t>
-  </si>
-  <si>
-    <t>None (Passive)</t>
-  </si>
-  <si>
-    <t>Enemy</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Đây là hiệu ứng </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lethal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Chạm là chết).</t>
-    </r>
-  </si>
-  <si>
-    <t>Aura/Global</t>
-  </si>
-  <si>
-    <t>Self</t>
-  </si>
-  <si>
-    <t>AddStats</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Cần một biến đếm toàn cục </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF444746"/>
-        <rFont val="Google Sans Text"/>
-        <family val="2"/>
-      </rPr>
-      <t>NilesSummonCount</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>Grrrr</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>Babylon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ereskigal </t>
+  </si>
+  <si>
+    <t>When you sell a Babylon unit, Consume it (3 times per turn)</t>
+  </si>
+  <si>
+    <t>Ninurta</t>
+  </si>
+  <si>
+    <t>After you deploy 3 units, increase your Income by 1 coin next turn</t>
+  </si>
+  <si>
+    <t>Utu</t>
+  </si>
+  <si>
+    <t>After you deploy a Babylon unit, give all allies +1/+1 (increases by +1/+1 after you deploy 3 Babylon Units)</t>
+  </si>
+  <si>
+    <t>Ki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When you deploy a Babylon unit, give it  +3/+3 (increase by +2/+2 for each unit deployed this turn) </t>
+  </si>
+  <si>
+    <t>Nanna</t>
+  </si>
+  <si>
+    <t>When you sell this, give this stats to 2 random Babylon ally</t>
+  </si>
+  <si>
+    <t>Ashur</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Whenever you sell a Unit, give all allies +5/+5 </t>
+  </si>
+  <si>
+    <t>Enki</t>
+  </si>
+  <si>
+    <t>Taunt; khi bị tấn công: phản lại atk của kẻ tấn công</t>
+  </si>
+  <si>
+    <t>Gugalana</t>
+  </si>
+  <si>
+    <t>Taunt; After you deploy this, Trible its stats</t>
+  </si>
+  <si>
+    <t>Umu  Drabutu</t>
+  </si>
+  <si>
+    <t>Deploy: Get 2 random babylon Unit</t>
+  </si>
+  <si>
+    <t>Enkidu</t>
+  </si>
+  <si>
+    <t>After you deploy a babylon unit, give this and the ally on the right +3/+3</t>
+  </si>
+  <si>
+    <t>Gilgamesh</t>
+  </si>
+  <si>
+    <t>Whenever this gain stats, add +3/+2 to that amount.</t>
+  </si>
+  <si>
+    <t>Humbaba</t>
+  </si>
+  <si>
+    <t>Slay: get 2 coin</t>
+  </si>
+  <si>
+    <t>Asag</t>
+  </si>
+  <si>
+    <t>Deploy: double state 1 random unit</t>
+  </si>
+  <si>
+    <t>Usumgallu</t>
+  </si>
+  <si>
+    <t>Taunt; bị tấn công: +1/+2 cho tất cả babylon unit</t>
+  </si>
+  <si>
+    <t>Lamashtu</t>
+  </si>
+  <si>
+    <t>when buy a babylon, +1 atk all babylon unit</t>
+  </si>
+  <si>
+    <t>Pazuzu</t>
+  </si>
+  <si>
+    <t>Deploy: get 2 coin</t>
+  </si>
+  <si>
+    <t>Kingu</t>
+  </si>
+  <si>
+    <t>Taunt; reborn</t>
+  </si>
+  <si>
+    <t>Uridimmu</t>
+  </si>
+  <si>
+    <t>when buy a babylon, +1 hp all babylon unit</t>
+  </si>
+  <si>
+    <t>Ugallu</t>
+  </si>
+  <si>
+    <t>when you sell this, get 1 ramdom Babylon unit</t>
+  </si>
+  <si>
+    <t>Kusarikku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After you sell a Babylon unit, gain +1/+1 </t>
+  </si>
+  <si>
+    <t>Babilonian Soldier</t>
+  </si>
+  <si>
+    <t>After you deploy a Babylon unit, gain +1 hp</t>
+  </si>
+  <si>
+    <t>Sumerian Scholar</t>
+  </si>
+  <si>
+    <t>deploy: get 1 coin</t>
+  </si>
+  <si>
+    <t>spell-art_01</t>
+  </si>
+  <si>
+    <t>spell-art_02</t>
+  </si>
+  <si>
+    <t>spell-art_03</t>
+  </si>
+  <si>
+    <t>spell-art_04</t>
+  </si>
+  <si>
+    <t>spell-art_05</t>
+  </si>
+  <si>
+    <t>spell-art_06</t>
+  </si>
+  <si>
+    <t>spell-art_07</t>
+  </si>
+  <si>
+    <t>spell-art_08</t>
+  </si>
+  <si>
+    <t>spell-art_09</t>
+  </si>
+  <si>
+    <t>spell-art_10</t>
+  </si>
+  <si>
+    <t>spell-art_11</t>
+  </si>
+  <si>
+    <t>spell-art_12</t>
+  </si>
+  <si>
+    <t>spell-art_13</t>
+  </si>
+  <si>
+    <t>spell-art_14</t>
+  </si>
+  <si>
+    <t>spell-art_16</t>
+  </si>
+  <si>
+    <t>spell-art_17</t>
+  </si>
+  <si>
+    <t>spell-art_18</t>
+  </si>
+  <si>
+    <t>spell-art_19</t>
+  </si>
+  <si>
+    <t>spell-art_20</t>
+  </si>
+  <si>
+    <t>spell-art_21</t>
+  </si>
+  <si>
+    <t>spell-art_22</t>
+  </si>
+  <si>
+    <t>spell-art_23</t>
+  </si>
+  <si>
+    <t>spell-art_24</t>
+  </si>
+  <si>
+    <t>Gain 1 coin</t>
+  </si>
+  <si>
+    <t>Give a unit +3 Attack</t>
+  </si>
+  <si>
+    <t>Give a unit +3 Health and Taunt</t>
+  </si>
+  <si>
+    <t>FileName</t>
+  </si>
+  <si>
+    <t>Ancient Coin</t>
+  </si>
+  <si>
+    <t>Sharpen Blade</t>
+  </si>
+  <si>
+    <t>Plated Armor</t>
+  </si>
+  <si>
+    <t>Quick Recruit</t>
+  </si>
+  <si>
+    <t>Get a random Tier 1 unit</t>
+  </si>
+  <si>
+    <t>Sanctum Heist</t>
+  </si>
+  <si>
+    <t>Take a random unit from the current Shop</t>
+  </si>
+  <si>
+    <t>Let's Feast</t>
+  </si>
+  <si>
+    <t>Balance Stance</t>
+  </si>
+  <si>
+    <t>Give a unit +2/+2</t>
+  </si>
+  <si>
+    <t>Trader's Trick</t>
+  </si>
+  <si>
+    <t>Increase your Income by 2 until next turn</t>
+  </si>
+  <si>
+    <t>Tailored Recruit</t>
+  </si>
+  <si>
+    <t>Get a different unit from the same Realm</t>
+  </si>
+  <si>
+    <t>Divine Inspiration</t>
+  </si>
+  <si>
+    <t>Give a unit stats equal to the Shop's Tier</t>
+  </si>
+  <si>
+    <t>Caishen's Knock</t>
+  </si>
+  <si>
+    <t>Increase your Income by 1 permanently</t>
+  </si>
+  <si>
+    <t>Give 3 allies in board +1 health</t>
+  </si>
+  <si>
+    <t>Strengthen Bond</t>
+  </si>
+  <si>
+    <t>Give all allies +1/+1</t>
+  </si>
+  <si>
+    <t>Rising Spirit</t>
+  </si>
+  <si>
+    <t>Battle Cry</t>
+  </si>
+  <si>
+    <t>Give a unit "EndTurnShop, gain +2/+2"</t>
+  </si>
+  <si>
+    <t>Give a unit "StartOfBattle, gain all allies +2/+1"</t>
+  </si>
+  <si>
+    <t>Wager</t>
+  </si>
+  <si>
+    <t>If you win your next battle, gain 3 coin</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,23 +524,10 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF444746"/>
-      <name val="Google Sans Text"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -408,7 +538,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -416,40 +546,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -785,12 +888,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8F2931-AC64-4BC6-B604-4088002CBEDE}">
   <dimension ref="A1:P24"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -810,7 +913,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -830,7 +933,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -850,7 +953,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -870,7 +973,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -890,7 +993,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -910,7 +1013,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -930,7 +1033,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -950,7 +1053,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -970,7 +1073,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -990,7 +1093,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1010,7 +1113,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1030,10 +1133,10 @@
         <v>40</v>
       </c>
       <c r="P12" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1053,7 +1156,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -1073,7 +1176,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1093,7 +1196,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1113,7 +1216,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1133,7 +1236,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -1153,7 +1256,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -1173,7 +1276,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -1193,7 +1296,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -1213,7 +1316,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -1233,7 +1336,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -1249,8 +1352,11 @@
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="F23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -1265,6 +1371,9 @@
       </c>
       <c r="E24">
         <v>2</v>
+      </c>
+      <c r="F24" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1274,120 +1383,801 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99BC0751-DD6C-4B8D-A53C-C1976B6374A6}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A2" s="2" t="s">
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+      <c r="F10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12">
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A3" s="2" t="s">
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="42" thickBot="1">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>74</v>
+      <c r="E14">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>5</v>
+      </c>
+      <c r="F16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B73F56F-5235-4F16-9AAD-8ACFD5C0A7B7}">
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E12" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" t="s">
+        <v>146</v>
+      </c>
+      <c r="G13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" t="s">
+        <v>147</v>
+      </c>
+      <c r="E14" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" t="s">
+        <v>148</v>
+      </c>
+      <c r="E15" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>0</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bản sao trước update giao diện
</commit_message>
<xml_diff>
--- a/Assets/Document/02_Data/a_CardsData.xlsx
+++ b/Assets/Document/02_Data/a_CardsData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspaces\specialized-essays\AutoChess\Assets\Document\02_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DEF3E5-C938-4188-ADE3-EE4FEB83D547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14434B6E-5D9F-49AE-A3BD-919B10776461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{4D4D67B0-B191-4148-8DB5-7E5E04C9AFB3}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="162">
   <si>
     <t>Tribe</t>
   </si>
@@ -397,18 +397,6 @@
     <t>spell-art_20</t>
   </si>
   <si>
-    <t>spell-art_21</t>
-  </si>
-  <si>
-    <t>spell-art_22</t>
-  </si>
-  <si>
-    <t>spell-art_23</t>
-  </si>
-  <si>
-    <t>spell-art_24</t>
-  </si>
-  <si>
     <t>Gain 1 coin</t>
   </si>
   <si>
@@ -448,9 +436,6 @@
     <t>Balance Stance</t>
   </si>
   <si>
-    <t>Give a unit +2/+2</t>
-  </si>
-  <si>
     <t>Trader's Trick</t>
   </si>
   <si>
@@ -460,9 +445,6 @@
     <t>Tailored Recruit</t>
   </si>
   <si>
-    <t>Get a different unit from the same Realm</t>
-  </si>
-  <si>
     <t>Divine Inspiration</t>
   </si>
   <si>
@@ -475,9 +457,6 @@
     <t>Increase your Income by 1 permanently</t>
   </si>
   <si>
-    <t>Give 3 allies in board +1 health</t>
-  </si>
-  <si>
     <t>Strengthen Bond</t>
   </si>
   <si>
@@ -487,15 +466,9 @@
     <t>Rising Spirit</t>
   </si>
   <si>
-    <t>Battle Cry</t>
-  </si>
-  <si>
     <t>Give a unit "EndTurnShop, gain +2/+2"</t>
   </si>
   <si>
-    <t>Give a unit "StartOfBattle, gain all allies +2/+1"</t>
-  </si>
-  <si>
     <t>Wager</t>
   </si>
   <si>
@@ -503,6 +476,57 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Devil's Deal</t>
+  </si>
+  <si>
+    <t>Ritual of the Realm</t>
+  </si>
+  <si>
+    <t>Olympic Flame</t>
+  </si>
+  <si>
+    <t>Give a unit Double Atk state and Safeguard</t>
+  </si>
+  <si>
+    <t>Change of Heart</t>
+  </si>
+  <si>
+    <t>Give a unit Taunt and +5 Health. If it already has Taunt, remove Taunt and give it +3 Attack</t>
+  </si>
+  <si>
+    <t>Military Support</t>
+  </si>
+  <si>
+    <t>Get  3 ramdom Tier 5 units</t>
+  </si>
+  <si>
+    <t>spell-art_15</t>
+  </si>
+  <si>
+    <t>Coin</t>
+  </si>
+  <si>
+    <t>Gate of Destruction</t>
+  </si>
+  <si>
+    <t>Remove a Unit. Give its stats to a random ally</t>
+  </si>
+  <si>
+    <t>Give 3 allies in board +2 health</t>
+  </si>
+  <si>
+    <t>Give a unit +3/+3</t>
+  </si>
+  <si>
+    <t>Lose a Life, then gain 6 coin</t>
+  </si>
+  <si>
+    <t>Choose a unit, give a unit from the same Realm up 1 Tier</t>
+  </si>
+  <si>
+    <t>Choose a unit,  get a different unit from the same Realm</t>
   </si>
 </sst>
 </file>
@@ -1854,14 +1878,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B73F56F-5235-4F16-9AAD-8ACFD5C0A7B7}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="4" width="17.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.5546875" customWidth="1"/>
+    <col min="4" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1869,311 +1893,421 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>99</v>
-      </c>
-      <c r="D2" t="s">
-        <v>126</v>
       </c>
       <c r="E2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>100</v>
-      </c>
-      <c r="D3" t="s">
-        <v>127</v>
       </c>
       <c r="E3" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>0</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
         <v>101</v>
-      </c>
-      <c r="D4" t="s">
-        <v>128</v>
       </c>
       <c r="E4" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
         <v>102</v>
       </c>
-      <c r="D5" t="s">
-        <v>129</v>
-      </c>
       <c r="E5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+      <c r="F5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
         <v>103</v>
       </c>
-      <c r="D6" t="s">
-        <v>131</v>
-      </c>
       <c r="E6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+      <c r="F6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
         <v>104</v>
       </c>
-      <c r="D7" t="s">
-        <v>133</v>
-      </c>
       <c r="E7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>0</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
         <v>105</v>
       </c>
-      <c r="D8" t="s">
-        <v>134</v>
-      </c>
       <c r="E8" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+      <c r="F8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>0</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
         <v>106</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" t="s">
+        <v>145</v>
+      </c>
+      <c r="F11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" t="s">
         <v>136</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F13" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>1</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E14" t="s">
         <v>138</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F14" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>3</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11" t="s">
-        <v>108</v>
-      </c>
-      <c r="D11" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" t="s">
         <v>140</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F15" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>1</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>109</v>
-      </c>
-      <c r="D12" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>153</v>
+      </c>
+      <c r="E16" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>0</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" t="s">
         <v>142</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F18" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>1</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D13" t="s">
-        <v>145</v>
-      </c>
-      <c r="E13" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+      <c r="E19" t="s">
         <v>146</v>
       </c>
-      <c r="G13" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14">
-        <v>3</v>
-      </c>
-      <c r="C14" t="s">
-        <v>111</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="F19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" t="s">
         <v>147</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15">
-        <v>3</v>
-      </c>
-      <c r="C15" t="s">
-        <v>112</v>
-      </c>
-      <c r="D15" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>0</v>
-      </c>
-      <c r="B17">
-        <v>3</v>
-      </c>
-      <c r="C17" t="s">
-        <v>113</v>
-      </c>
-      <c r="D17" t="s">
-        <v>151</v>
-      </c>
-      <c r="E17" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C19" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C20" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C21" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C22" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C25" t="s">
-        <v>121</v>
+    <row r="49" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I49" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>